<commit_message>
Change data field to "niveau scolaire"
</commit_message>
<xml_diff>
--- a/5-excel-analysis/data_fr.xlsx
+++ b/5-excel-analysis/data_fr.xlsx
@@ -22,19 +22,19 @@
     <t>le nom de l’école</t>
   </si>
   <si>
+    <t>le type de l’école</t>
+  </si>
+  <si>
     <t>niveau scolaire</t>
   </si>
   <si>
-    <t>le niveau de l’école</t>
-  </si>
-  <si>
     <t>la langue de l’école</t>
   </si>
   <si>
     <t>la ville</t>
   </si>
   <si>
-    <t>inscription</t>
+    <t>l’effectif</t>
   </si>
   <si>
     <t xml:space="preserve">le pourcentage d’élèves bénéficiaires de services d’éducation de l’enfance en difficulté </t>
@@ -4152,7 +4152,7 @@
   <cols>
     <col min="1" max="1" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="4" width="12.43357142857143" customWidth="1" bestFit="1"/>

</xml_diff>

<commit_message>
Change data field to "inscription"
</commit_message>
<xml_diff>
--- a/5-excel-analysis/data_fr.xlsx
+++ b/5-excel-analysis/data_fr.xlsx
@@ -34,7 +34,7 @@
     <t>la ville</t>
   </si>
   <si>
-    <t>l’effectif</t>
+    <t>inscription</t>
   </si>
   <si>
     <t xml:space="preserve">le pourcentage d’élèves bénéficiaires de services d’éducation de l’enfance en difficulté </t>
@@ -3786,7 +3786,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3797,6 +3797,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -3833,10 +3839,10 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -4190,7 +4196,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -4219,7 +4225,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -4248,7 +4254,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -4277,7 +4283,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -4306,7 +4312,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -4335,7 +4341,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -4364,7 +4370,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -4393,7 +4399,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -4422,7 +4428,7 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -4451,7 +4457,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -4480,7 +4486,7 @@
         <v>43</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -4509,7 +4515,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
@@ -4538,7 +4544,7 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -4567,7 +4573,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -4596,7 +4602,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1" t="s">
         <v>9</v>
       </c>
@@ -4625,7 +4631,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
@@ -4654,7 +4660,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -4683,7 +4689,7 @@
         <v>59</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="1" t="s">
         <v>9</v>
       </c>
@@ -4712,7 +4718,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -4741,7 +4747,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
@@ -4770,7 +4776,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
@@ -4799,7 +4805,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="1" t="s">
         <v>9</v>
       </c>
@@ -4828,7 +4834,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -4857,7 +4863,7 @@
         <v>72</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="1" t="s">
         <v>9</v>
       </c>
@@ -4886,7 +4892,7 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="1" t="s">
         <v>9</v>
       </c>
@@ -4915,7 +4921,7 @@
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="1" t="s">
         <v>9</v>
       </c>
@@ -4944,7 +4950,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="1" t="s">
         <v>9</v>
       </c>
@@ -4973,7 +4979,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="1" t="s">
         <v>9</v>
       </c>
@@ -5002,7 +5008,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="1" t="s">
         <v>9</v>
       </c>
@@ -5031,7 +5037,7 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="1" t="s">
         <v>9</v>
       </c>

</xml_diff>